<commit_message>
Update CoralBean and Geiger
</commit_message>
<xml_diff>
--- a/data/PSBP_Master_Plant_Signage.xlsx
+++ b/data/PSBP_Master_Plant_Signage.xlsx
@@ -3562,8 +3562,7 @@
       </c>
       <c r="Z11" s="33" t="inlineStr">
         <is>
-          <t>Geiger Tree
-Sebesten Plum (for fruit)</t>
+          <t>Scarlet Cordia · Sebesten Plum (for fruit)</t>
         </is>
       </c>
       <c r="AA11" s="33" t="inlineStr">
@@ -4276,10 +4275,10 @@
       <c r="H16" s="32" t="n"/>
       <c r="I16" s="33" t="inlineStr">
         <is>
-          <t>The scarlet tubular flowers of Coral Bean are timed almost perfectly to coincide with the spring migration of Ruby-throated Hummingbirds moving north along the Gulf Coast — making this one of the most ecologically timed native plants in the park.
-The brilliant red seeds that follow are beautiful, familiar-looking, and seriously toxic.
-Thorny, deciduous, and tough enough to grow in pure sand and salt spray.
-A genuine Florida native that earns its keep for wildlife year-round.</t>
+          <t>The scarlet tubular flowers bloom in step with the spring migration of **Ruby-throated Hummingbirds** moving north along the Gulf Coast.
+The brilliant red seeds that follow are beautiful, familiar-looking, and **seriously toxic**.
+Thorny, deciduous, and tough enough to grow in pure sand and **salt spray**.
+A true **Florida native** that provides year-round value for wildlife.</t>
         </is>
       </c>
       <c r="J16" s="33" t="inlineStr">
@@ -4293,12 +4292,12 @@
 The seeds are among the most deceptively dangerous in Florida. They look like polished red beads — and have historically been used exactly that way, strung into jewelry and decorations across the Caribbean and Gulf South. They contain a suite of toxic alkaloids including erysopine, erythrinine, and hypaphorine, known to cause paralysis when ingested. In Mexico the seeds have been used as rat poison. Handle with gloves; keep away from children.
 Despite its toxicity, the Cherokee people used root decoctions medicinally for kidney and urinary conditions, and Florida Ethnobotany devotes two full pages to traditional uses of this plant across Indigenous cultures of the Southeast.
 The name herbacea — Latin for 'herbaceous' or 'low-growing' — was given because this species is more shrubby than the large tropical Erythrina trees common in South America and Africa, some of which reach 100 feet and are used as shade trees for coffee and cacao plantations. This is the modest North American representative of a globally significant genus.
-A member of the Fabaceae family — the same legume family as Sunshine Mimosa, Royal Poinciana, and Peacock Flower also in the park. The genus name Erythrina comes from the Greek erythros, meaning red — a reference to the flowers and seeds that define the plant.</t>
+A member of the Fabaceae family — the same legume family as Sunshine Mimosa, Royal Poinciana, and Dwarf Poinciana also in the park. The genus name Erythrina comes from the Greek erythros, meaning red — a reference to the flowers and seeds that define the plant.</t>
         </is>
       </c>
       <c r="L16" s="33" t="inlineStr">
         <is>
-          <t>The Coral Bean is one of the most hummingbird-focused native plants in Florida. Its long scarlet tubular flowers are shaped specifically for hummingbird bills and timed to coincide with Ruby-throated Hummingbird migration in spring — feeding northbound birds at a critical moment in their journey. Butterflies with longer tongues and bumblebees also work the flowers. The brilliant red seeds that follow are dispersed by birds that carry them from the split pods. The plant's thorny stems and dense branching habit make it an ideal refuge for small birds seeking protected roosting and nesting cover. The Erythrina borer moth (Terastia meticulosalis) uses it as a larval host — a less glamorous but ecologically real wildlife relationship.</t>
+          <t>The Coral Bean is one of the most hummingbird-focused native plants in Florida. Its long scarlet tubular flowers are shaped specifically for hummingbird bills and timed to coincide with Ruby-throated Hummingbird migration in spring — feeding northbound birds at a critical moment in their journey. Butterflies with longer tongues and bumblebees also work the flowers. The brilliant red seeds that follow are dispersed by birds that carry them from the split pods. The plant's thorny stems and dense branching habit make it an ideal refuge for small birds seeking protected roosting and nesting cover. The Erythrina borer moth (Terastia meticulosalis) uses it as a larval host.</t>
         </is>
       </c>
       <c r="M16" s="33" t="inlineStr">
@@ -4309,7 +4308,7 @@
 Seeds: Brilliant coral-red, polished-looking. TOXIC — contain multiple alkaloids causing paralysis. Handle with gloves.
 Leaves: Compound, with three deltoid (arrowhead-shaped) light green leaflets, each with tiny prickles along the underside of the margin. Stems armed with short curved spines.
 Bark: Smooth, light gray to whitish on mature stems.
-What to Look For: In spring, watch for vivid scarlet flower spikes appearing on nearly bare branches — and watch those branches for hummingbirds. In fall and winter, the split bean pods displaying brilliant red seeds against bare stems are unmistakable. Run a careful finger along a leaflet margin to feel the fine prickles — a reliable tactile ID feature.</t>
+What to Look For: In spring, watch for vivid scarlet flower spikes appearing on nearly bare branches — and watch those branches for hummingbirds. In fall and winter, the split bean pods displaying brilliant red seeds against bare stems are easy to spot. Run a careful finger along a leaflet margin to feel the fine prickles — a reliable tactile ID feature.</t>
         </is>
       </c>
       <c r="N16" s="33" t="inlineStr">

</xml_diff>